<commit_message>
Update Excell for Student Awards
</commit_message>
<xml_diff>
--- a/excell/MWSCAS_Student_Paper_Awards.xlsx
+++ b/excell/MWSCAS_Student_Paper_Awards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MWSCAS Web Site\2026-08 MWSCAS Web Site\MWSCAS_GitHub_Beta5\Student Paper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{386F6024-D548-436C-9468-0F5B9540F35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60CEACDD-F8B3-4125-806C-BEE2B5D8565D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="305">
   <si>
     <t>Year</t>
   </si>
@@ -913,6 +913,30 @@
   </si>
   <si>
     <t>Pukar Malla, Hasnain Lakdawala, Kevin Kornegay, and Krishnamurthy Soumyanath</t>
+  </si>
+  <si>
+    <t>Siyuan Yu</t>
+  </si>
+  <si>
+    <t>Yuting Shen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valentin Poisson </t>
+  </si>
+  <si>
+    <t>Eindhoven University of Technology, Netherlands</t>
+  </si>
+  <si>
+    <t>CEA-LETI, University of Grenoble, France</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A 1 micro Watt Activity-Aware Asynchronous Delta Modulator with Animated Dual Mode Operation </t>
+  </si>
+  <si>
+    <t>2.2 fJ/Conversion-Step 9.74-ENOB 10 MS/s SAR ADC with 1.5×Input Range Global System Optimization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A 2-Stage EM Algorithm for Online Peak Detection, an Application to TCSPC Data </t>
   </si>
 </sst>
 </file>
@@ -1262,7 +1286,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="78.1796875" customWidth="1"/>
@@ -2650,42 +2674,51 @@
       <c r="A83" s="1" t="s">
         <v>256</v>
       </c>
+      <c r="B83" s="1">
+        <v>1</v>
+      </c>
       <c r="C83" t="s">
-        <v>255</v>
+        <v>297</v>
+      </c>
+      <c r="D83" t="s">
+        <v>283</v>
+      </c>
+      <c r="E83" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B84" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C84" t="s">
-        <v>259</v>
+        <v>298</v>
       </c>
       <c r="D84" t="s">
-        <v>266</v>
+        <v>300</v>
       </c>
       <c r="E84" t="s">
-        <v>260</v>
+        <v>303</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B85" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C85" t="s">
-        <v>261</v>
-      </c>
-      <c r="D85" t="s">
-        <v>265</v>
+        <v>299</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>301</v>
       </c>
       <c r="E85" t="s">
-        <v>262</v>
+        <v>304</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
@@ -2693,74 +2726,108 @@
         <v>257</v>
       </c>
       <c r="B86" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C86" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="D86" t="s">
         <v>266</v>
       </c>
       <c r="E86" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B87" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C87" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="D87" t="s">
         <v>265</v>
       </c>
       <c r="E87" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B88" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C88" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="D88" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="E88" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>258</v>
       </c>
       <c r="B89" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C89" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="D89" t="s">
-        <v>275</v>
-      </c>
-      <c r="E89" s="2" t="s">
-        <v>274</v>
+        <v>265</v>
+      </c>
+      <c r="E89" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B90" s="1">
+        <v>2</v>
+      </c>
+      <c r="C90" t="s">
+        <v>270</v>
+      </c>
+      <c r="D90" t="s">
+        <v>272</v>
+      </c>
+      <c r="E90" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A91" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B91" s="1">
+        <v>3</v>
+      </c>
+      <c r="C91" t="s">
+        <v>273</v>
+      </c>
+      <c r="D91" t="s">
+        <v>275</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A92" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="C90" t="s">
+      <c r="C92" t="s">
         <v>255</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Student Paper Awards 2026
</commit_message>
<xml_diff>
--- a/excell/MWSCAS_Student_Paper_Awards.xlsx
+++ b/excell/MWSCAS_Student_Paper_Awards.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MWSCAS Web Site\2026-08 MWSCAS Web Site\MWSCAS_GitHub_Beta5\Student Paper\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MWSCAS Web Site\2026-08 MWSCAS Web Site\MWSCAS_GitHub_Beta5\Student Paper Awards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60CEACDD-F8B3-4125-806C-BEE2B5D8565D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24E91708-F766-47D2-83A3-1E8702BE4655}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="327">
   <si>
     <t>Year</t>
   </si>
@@ -937,6 +937,73 @@
   </si>
   <si>
     <t xml:space="preserve">A 2-Stage EM Algorithm for Online Peak Detection, an Application to TCSPC Data </t>
+  </si>
+  <si>
+    <t>Introduction</t>
+  </si>
+  <si>
+    <t>MWSCAS Student Paper Contest Winners</t>
+  </si>
+  <si>
+    <t>1-C</t>
+  </si>
+  <si>
+    <t>Jacob O'Donnell, Elaine Greenfield, Hagar Hendy, Karsten Bergthold, Cory Merkel and Tejasvi Das</t>
+  </si>
+  <si>
+    <t>Evaluating FeFET and Memristor Performance in Time-Domain Computing Applications</t>
+  </si>
+  <si>
+    <t>Rochester Institute of Technology, Rochester, NY, USA</t>
+  </si>
+  <si>
+    <t>A 24.5-To-40.5 GHz 6-Bit Vector Modulator for Mm-Wave 5G Beamformers</t>
+  </si>
+  <si>
+    <t>Cairo University, Giza, Egypt</t>
+  </si>
+  <si>
+    <t>Jongchan Pyeon, Rudra Biswas, Mehdi Kiani, Farnaz Tehranchi</t>
+  </si>
+  <si>
+    <t>A Deep Learning Framework for Predicting Ultrasound Array Geometry and Skull Shape in Precision Ultrasound Neuromodulation</t>
+  </si>
+  <si>
+    <t>The Pennsylvania State University, University Park, PA, USA</t>
+  </si>
+  <si>
+    <t>The first MWSCAS Student Paper Contest was held at the 1997 IEEE International Midwest Symposium on Circuits and Systems in Sacramento, California. Conference Chair Michael A. Soderstrand introduced the contest as a way to attract more students to the conference by soliciting a large number of paper submissions in which a student was the primary author. Ten papers were then selected by the conference’s Student Paper Award Committee for presentation in a special Student Paper Contest session, which was featured prominently at the symposium. The response exceeded all expectations: the committee selected ten papers from nearly 200 submissions. The resulting contest became one of the highlights of the 1997 conference and has continued as an integral part of every MWSCAS conference since 1997.
+The following table lists the MWSCAS Student Paper Contest award recipients:</t>
+  </si>
+  <si>
+    <t>Mohamed Saad Aly, Mohamed A. Y. Abdalla, and Mohamed Salah Mobarak</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>Noah Michels</t>
+  </si>
+  <si>
+    <t>Tomoro M. Jones</t>
+  </si>
+  <si>
+    <t>Lexie Drackley</t>
+  </si>
+  <si>
+    <t>Kyushu Institute of Technology, Kitakyushu, Fukuoka, Japan</t>
+  </si>
+  <si>
+    <t>University of Michigan, Ann Arbor, MI, USA</t>
+  </si>
+  <si>
+    <t>A Novel Differential AC-AC Charge Pump Surpassing the Fibonacci Gain Per Capacitor Limit</t>
+  </si>
+  <si>
+    <t>An Updatable Nonvolatile Multi-Bit Memory Array Core for Compute-In-Memory Architectures</t>
+  </si>
+  <si>
+    <t>Passive ED Modeling and Temperature Characterization of an ED-First Wake-Up Receiver</t>
   </si>
 </sst>
 </file>
@@ -1286,63 +1353,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E92"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="78.1796875" customWidth="1"/>
+    <col min="3" max="3" width="81.54296875" customWidth="1"/>
     <col min="4" max="4" width="83.6328125" customWidth="1"/>
     <col min="5" max="5" width="117.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
+        <v>305</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="159.5" x14ac:dyDescent="0.35">
       <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
+        <v>306</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -1350,84 +1399,84 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
         <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -1435,50 +1484,50 @@
         <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="E10" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="D11" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="E11" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -1486,16 +1535,16 @@
         <v>35</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E12" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -1503,16 +1552,16 @@
         <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="E13" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -1520,16 +1569,16 @@
         <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="E14" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -1537,16 +1586,16 @@
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E15" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -1554,16 +1603,16 @@
         <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="D16" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="E16" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -1571,50 +1620,50 @@
         <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="D17" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="E17" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="E18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="C19" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E19" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -1622,50 +1671,50 @@
         <v>67</v>
       </c>
       <c r="B20" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C20" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D20" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E20" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="C21" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="D21" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="E21" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D22" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E22" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
@@ -1673,16 +1722,16 @@
         <v>76</v>
       </c>
       <c r="B23" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C23" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D23" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="E23" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
@@ -1690,16 +1739,16 @@
         <v>76</v>
       </c>
       <c r="B24" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="C24" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D24" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="E24" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
@@ -1707,16 +1756,16 @@
         <v>76</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="D25" t="s">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="E25" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
@@ -1724,16 +1773,16 @@
         <v>76</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="D26" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="E26" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
@@ -1741,58 +1790,58 @@
         <v>76</v>
       </c>
       <c r="B27" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="C27" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="D27" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="E27" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>99</v>
+        <v>76</v>
+      </c>
+      <c r="B28" t="s">
+        <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>255</v>
+        <v>92</v>
+      </c>
+      <c r="D28" t="s">
+        <v>93</v>
+      </c>
+      <c r="E28" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="B29" t="s">
-        <v>6</v>
+        <v>95</v>
       </c>
       <c r="C29" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="D29" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="E29" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>100</v>
-      </c>
-      <c r="B30" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="C30" t="s">
-        <v>104</v>
-      </c>
-      <c r="D30" t="s">
-        <v>105</v>
-      </c>
-      <c r="E30" t="s">
-        <v>106</v>
+        <v>255</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
@@ -1800,50 +1849,50 @@
         <v>100</v>
       </c>
       <c r="B31" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C31" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D31" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="E31" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B32" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="D32" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="E32" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B33" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C33" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="D33" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="E33" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
@@ -1851,50 +1900,50 @@
         <v>110</v>
       </c>
       <c r="B34" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C34" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D34" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="E34" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="B35" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C35" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D35" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="E35" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="B36" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C36" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="D36" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="E36" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
@@ -1902,50 +1951,50 @@
         <v>120</v>
       </c>
       <c r="B37" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C37" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D37" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E37" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B38" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D38" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="E38" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="B39" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C39" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="D39" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="E39" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
@@ -1953,50 +2002,50 @@
         <v>130</v>
       </c>
       <c r="B40" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C40" t="s">
-        <v>296</v>
+        <v>131</v>
       </c>
       <c r="D40" t="s">
-        <v>294</v>
+        <v>132</v>
       </c>
       <c r="E40" t="s">
-        <v>295</v>
+        <v>133</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B41" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D41" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="E41" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B42" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C42" t="s">
-        <v>141</v>
+        <v>296</v>
       </c>
       <c r="D42" t="s">
-        <v>142</v>
+        <v>294</v>
       </c>
       <c r="E42" t="s">
-        <v>143</v>
+        <v>295</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
@@ -2004,50 +2053,50 @@
         <v>137</v>
       </c>
       <c r="B43" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C43" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="D43" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="E43" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="B44" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C44" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="D44" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="E44" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="B45" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C45" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="D45" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="E45" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
@@ -2055,50 +2104,50 @@
         <v>147</v>
       </c>
       <c r="B46" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C46" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="D46" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E46" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="B47" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C47" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="D47" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="E47" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="B48" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C48" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="D48" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="E48" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
@@ -2106,50 +2155,50 @@
         <v>157</v>
       </c>
       <c r="B49" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C49" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="D49" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="E49" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B50" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C50" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="D50" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="E50" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B51" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C51" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="D51" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="E51" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
@@ -2157,50 +2206,50 @@
         <v>167</v>
       </c>
       <c r="B52" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C52" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D52" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="E52" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="B53" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="C53" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="D53" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="E53" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="B54" t="s">
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="C54" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="D54" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="E54" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
@@ -2208,16 +2257,16 @@
         <v>177</v>
       </c>
       <c r="B55" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C55" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="D55" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="E55" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
@@ -2225,50 +2274,50 @@
         <v>177</v>
       </c>
       <c r="B56" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="C56" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="D56" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="E56" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>190</v>
+        <v>177</v>
       </c>
       <c r="B57" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C57" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="D57" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="E57" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>190</v>
+        <v>177</v>
       </c>
       <c r="B58" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C58" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D58" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="E58" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
@@ -2276,16 +2325,16 @@
         <v>190</v>
       </c>
       <c r="B59" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C59" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="D59" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="E59" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
@@ -2293,84 +2342,84 @@
         <v>190</v>
       </c>
       <c r="B60" t="s">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="C60" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="D60" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="E60" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="B61" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C61" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="D61" t="s">
-        <v>169</v>
+        <v>198</v>
       </c>
       <c r="E61" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="B62" t="s">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="C62" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="D62" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="E62" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="B63" t="s">
         <v>6</v>
       </c>
       <c r="C63" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="D63" t="s">
-        <v>212</v>
+        <v>169</v>
       </c>
       <c r="E63" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="B64" t="s">
         <v>10</v>
       </c>
       <c r="C64" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="D64" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="E64" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
@@ -2378,50 +2427,50 @@
         <v>210</v>
       </c>
       <c r="B65" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C65" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="D65" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="E65" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="B66" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C66" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="D66" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="E66" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="B67" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C67" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="D67" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="E67" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
@@ -2429,16 +2478,16 @@
         <v>220</v>
       </c>
       <c r="B68" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="C68" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="D68" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="E68" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
@@ -2446,109 +2495,109 @@
         <v>220</v>
       </c>
       <c r="B69" t="s">
+        <v>10</v>
+      </c>
+      <c r="C69" t="s">
+        <v>224</v>
+      </c>
+      <c r="D69" t="s">
+        <v>225</v>
+      </c>
+      <c r="E69" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>220</v>
+      </c>
+      <c r="B70" t="s">
+        <v>52</v>
+      </c>
+      <c r="C70" t="s">
+        <v>227</v>
+      </c>
+      <c r="D70" t="s">
+        <v>228</v>
+      </c>
+      <c r="E70" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>220</v>
+      </c>
+      <c r="B71" t="s">
         <v>56</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C71" t="s">
         <v>230</v>
       </c>
-      <c r="D69" t="s">
+      <c r="D71" t="s">
         <v>231</v>
       </c>
-      <c r="E69" t="s">
+      <c r="E71" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="1">
-        <v>2017</v>
-      </c>
-      <c r="B70" s="1">
-        <v>1</v>
-      </c>
-      <c r="C70" t="s">
-        <v>237</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="E70" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A71" s="1">
-        <v>2017</v>
-      </c>
-      <c r="B71" s="1">
-        <v>2</v>
-      </c>
-      <c r="C71" t="s">
-        <v>240</v>
-      </c>
-      <c r="D71" t="s">
-        <v>241</v>
-      </c>
-      <c r="E71" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>2017</v>
       </c>
       <c r="B72" s="1">
+        <v>1</v>
+      </c>
+      <c r="C72" t="s">
+        <v>237</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="E72" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A73" s="1">
+        <v>2017</v>
+      </c>
+      <c r="B73" s="1">
+        <v>2</v>
+      </c>
+      <c r="C73" t="s">
+        <v>240</v>
+      </c>
+      <c r="D73" t="s">
+        <v>241</v>
+      </c>
+      <c r="E73" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A74" s="1">
+        <v>2017</v>
+      </c>
+      <c r="B74" s="1">
         <v>3</v>
       </c>
-      <c r="C72" t="s">
+      <c r="C74" t="s">
         <v>243</v>
       </c>
-      <c r="D72" t="s">
+      <c r="D74" t="s">
         <v>244</v>
       </c>
-      <c r="E72" t="s">
+      <c r="E74" t="s">
         <v>245</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A73" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="C73" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A74" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="B74" s="1">
-        <v>1</v>
-      </c>
-      <c r="C74" t="s">
-        <v>285</v>
-      </c>
-      <c r="D74" t="s">
-        <v>286</v>
-      </c>
-      <c r="E74" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="B75" s="1">
-        <v>2</v>
+        <v>233</v>
       </c>
       <c r="C75" t="s">
-        <v>288</v>
-      </c>
-      <c r="D75" t="s">
-        <v>289</v>
-      </c>
-      <c r="E75" t="s">
-        <v>290</v>
+        <v>255</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
@@ -2556,50 +2605,50 @@
         <v>234</v>
       </c>
       <c r="B76" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C76" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="D76" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="E76" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B77" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C77" t="s">
-        <v>246</v>
+        <v>288</v>
       </c>
       <c r="D77" t="s">
-        <v>247</v>
+        <v>289</v>
       </c>
       <c r="E77" t="s">
-        <v>248</v>
+        <v>290</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B78" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C78" t="s">
-        <v>249</v>
+        <v>291</v>
       </c>
       <c r="D78" t="s">
-        <v>250</v>
+        <v>292</v>
       </c>
       <c r="E78" t="s">
-        <v>251</v>
+        <v>293</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
@@ -2607,50 +2656,50 @@
         <v>235</v>
       </c>
       <c r="B79" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C79" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="D79" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="E79" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B80" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C80" t="s">
-        <v>276</v>
+        <v>249</v>
       </c>
       <c r="D80" t="s">
-        <v>277</v>
+        <v>250</v>
       </c>
       <c r="E80" t="s">
-        <v>278</v>
+        <v>251</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B81" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C81" t="s">
-        <v>279</v>
+        <v>252</v>
       </c>
       <c r="D81" t="s">
-        <v>280</v>
+        <v>253</v>
       </c>
       <c r="E81" t="s">
-        <v>281</v>
+        <v>254</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
@@ -2658,50 +2707,50 @@
         <v>236</v>
       </c>
       <c r="B82" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C82" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="D82" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="E82" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
       <c r="B83" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C83" t="s">
-        <v>297</v>
+        <v>279</v>
       </c>
       <c r="D83" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="E83" t="s">
-        <v>302</v>
+        <v>281</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
-        <v>256</v>
+        <v>236</v>
       </c>
       <c r="B84" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C84" t="s">
-        <v>298</v>
+        <v>282</v>
       </c>
       <c r="D84" t="s">
-        <v>300</v>
+        <v>283</v>
       </c>
       <c r="E84" t="s">
-        <v>303</v>
+        <v>284</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
@@ -2709,50 +2758,50 @@
         <v>256</v>
       </c>
       <c r="B85" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C85" t="s">
-        <v>299</v>
-      </c>
-      <c r="D85" s="2" t="s">
-        <v>301</v>
+        <v>297</v>
+      </c>
+      <c r="D85" t="s">
+        <v>283</v>
       </c>
       <c r="E85" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B86" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C86" t="s">
-        <v>259</v>
+        <v>298</v>
       </c>
       <c r="D86" t="s">
-        <v>266</v>
+        <v>300</v>
       </c>
       <c r="E86" t="s">
-        <v>260</v>
+        <v>303</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B87" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C87" t="s">
-        <v>261</v>
-      </c>
-      <c r="D87" t="s">
-        <v>265</v>
+        <v>299</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>301</v>
       </c>
       <c r="E87" t="s">
-        <v>262</v>
+        <v>304</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
@@ -2760,75 +2809,203 @@
         <v>257</v>
       </c>
       <c r="B88" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C88" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="D88" t="s">
         <v>266</v>
       </c>
       <c r="E88" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B89" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C89" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="D89" t="s">
         <v>265</v>
       </c>
       <c r="E89" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B90" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C90" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="D90" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="E90" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>258</v>
       </c>
       <c r="B91" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C91" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="D91" t="s">
-        <v>275</v>
-      </c>
-      <c r="E91" s="2" t="s">
-        <v>274</v>
+        <v>265</v>
+      </c>
+      <c r="E91" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B92" s="1">
+        <v>2</v>
+      </c>
+      <c r="C92" t="s">
+        <v>270</v>
+      </c>
+      <c r="D92" t="s">
+        <v>272</v>
+      </c>
+      <c r="E92" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A93" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B93" s="1">
+        <v>3</v>
+      </c>
+      <c r="C93" t="s">
+        <v>273</v>
+      </c>
+      <c r="D93" t="s">
+        <v>275</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A94" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="C92" t="s">
-        <v>255</v>
+      <c r="B94" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C94" t="s">
+        <v>308</v>
+      </c>
+      <c r="D94" t="s">
+        <v>310</v>
+      </c>
+      <c r="E94" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A95" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C95" t="s">
+        <v>317</v>
+      </c>
+      <c r="D95" t="s">
+        <v>312</v>
+      </c>
+      <c r="E95" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A96" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="C96" t="s">
+        <v>313</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="E96" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A97" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B97" s="1">
+        <v>1</v>
+      </c>
+      <c r="C97" t="s">
+        <v>319</v>
+      </c>
+      <c r="D97" t="s">
+        <v>323</v>
+      </c>
+      <c r="E97" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A98" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B98" s="1">
+        <v>2</v>
+      </c>
+      <c r="C98" t="s">
+        <v>320</v>
+      </c>
+      <c r="D98" t="s">
+        <v>322</v>
+      </c>
+      <c r="E98" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A99" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="B99" s="1">
+        <v>3</v>
+      </c>
+      <c r="C99" t="s">
+        <v>321</v>
+      </c>
+      <c r="D99" t="s">
+        <v>323</v>
+      </c>
+      <c r="E99" t="s">
+        <v>326</v>
       </c>
     </row>
   </sheetData>

</xml_diff>